<commit_message>
Kolumna zestawienia mówi o zakresie pytania, nie o prośbie o pieniądze
Nazwa "Czy pytam MKiDN" czytała się jako prośba o sfinansowanie danej
pozycji, a pismo prosi wyłącznie o wskazanie właściwego programu
i trybu, nie o środki. Kolumna nazywa się teraz "W zakresie pytania do
MKiDN", a pod tabelą stoi legenda: czym jest "tak", czym "nie" i że
pismo nie jest wnioskiem o dotację.

Tak samo poprawione dwa zdania w nocie, w tym to podające sumę
665 880 zł - podaję ją jako skalę zadania, nie jako kwotę wnioskowaną.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/zestawienie-zadania.xlsx
+++ b/zestawienie-zadania.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="59">
   <si>
     <t xml:space="preserve">Nagroda Konstela - zestawienie zadania: co, w którym roku, z czego i o co pytam</t>
   </si>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Planowane źródło</t>
   </si>
   <si>
-    <t xml:space="preserve">Czy pytam MKiDN</t>
+    <t xml:space="preserve">W zakresie pytania do MKiDN</t>
   </si>
   <si>
     <t xml:space="preserve">Plebiscyt na rozmowę: nabór, ocena, prowadzenie</t>
@@ -185,6 +185,18 @@
   </si>
   <si>
     <t xml:space="preserve">Pozycje opisane jako "do wyceny" nie wchodzą do sum powyżej; ich wycena powstanie przed złożeniem wniosku.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Co oznacza kolumna "W zakresie pytania do MKiDN"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pismo nie jest wnioskiem o dotację i nie zawiera prośby o żadną z kwot wymienionych w tabeli.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"tak" - pozycja należy do części artystycznej przedsięwzięcia, której dotyczy pytanie o właściwy Program Ministra i o drogę finansowania. Jest to pytanie o tryb, nie o środki.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"nie" - pozycja jest poza tym pytaniem i ma być finansowana ze źródeł prywatnych. Wymieniam ją, aby było widoczne, że o tę samą pozycję nie zwracam się jednocześnie do dwóch źródeł.</t>
   </si>
 </sst>
 </file>
@@ -195,7 +207,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#\ ##,000&quot; zł&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,6 +272,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -318,16 +337,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -343,7 +366,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -355,23 +378,27 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -627,353 +654,373 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="7" t="n">
         <v>511996.8</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="7" t="n">
         <v>35168</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="7" t="n">
         <v>292422</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="7" t="n">
         <v>160160</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="7" t="n">
         <v>99600</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="F10" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="7" t="n">
         <v>75000</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="7" t="n">
         <v>80000</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D13" s="8" t="s">
+      <c r="D13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="7" t="n">
         <v>154480</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="F14" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
+    <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="8" t="s">
+      <c r="D15" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="F15" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D16" s="8" t="s">
+      <c r="D16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="7" t="n">
         <v>256800</v>
       </c>
-      <c r="E17" s="4" t="s">
+      <c r="E17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="F17" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="8" t="s">
+      <c r="D19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">SUMIFS(D6:D19,F6:F19,"tak")</f>
         <v>665880</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="D22" s="12" t="n">
+      <c r="D22" s="13" t="n">
         <f aca="false">SUM(D6:D19)</f>
         <v>1665626.8</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="14" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kwoty w zestawieniu z polskim separatorem tysięcy
Kod formatu zawierał spację i przecinek dosłownie, więc separator
tysięcy nie działał i kwota wyglądała jak "1 60160 zł". Format ma
teraz wymuszoną polską lokalizację, więc "160 160,00 zł" pokaże się
tak samo niezależnie od ustawień arkusza u odbiorcy.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WR2JsPawQK6ge7oAFtsinp
</commit_message>
<xml_diff>
--- a/zestawienie-zadania.xlsx
+++ b/zestawienie-zadania.xlsx
@@ -205,7 +205,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="#\ ##,000&quot; zł&quot;"/>
+    <numFmt numFmtId="165" formatCode="[$-415]#,##0.00&quot; zł&quot;"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1003,22 +1003,22 @@
         <v>54</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
         <v>58</v>
       </c>

</xml_diff>